<commit_message>
Fix practice challenge 2 readiness week and rebuild planner
Challenge 2 ("A small door, and one sentence from the Queen") covers
RHCSA-9.2 (password ageing), which is taught in Week 4, not Week 3.
The challenge itself requires setting password ageing parameters,
so it cannot be attempted until Week 4.

- practice.md: Changed challenge 2 readiness from week 3 to week 4
- planner/build.py: Changed challenge 2 week from 3 to 4
- planner/ict257-study-planner.xlsx: Rebuilt from updated build.py
- lessons.md: Pending changes from previous session (RHCSA-9.2 moved
  to Week 4, example link updated)
</commit_message>
<xml_diff>
--- a/planner/ict257-study-planner.xlsx
+++ b/planner/ict257-study-planner.xlsx
@@ -3136,11 +3136,11 @@
       </c>
       <c r="C6" s="30" t="inlineStr">
         <is>
-          <t>week 3</t>
+          <t>week 4</t>
         </is>
       </c>
       <c r="D6" s="22">
-        <f>SemesterStart+7*(3-1)</f>
+        <f>SemesterStart+7*(4-1)</f>
         <v/>
       </c>
       <c r="E6" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Reconcile the week 1 sections, the admin count and the planner weeks
The week 1 table cited RH124 0A.01 and 0A.02, a prefix used nowhere
else. The sequencing notes, coverage.md and the planner all say the
week keeps 00.02 and 00.03, so the table now says that too.

The course administration row counted 4 sections where coverage.md
lists 6 (three pairs, one per course). The page count still wants
checking against the courseware next semester.

coverage.md now says plainly that the Not mapped column includes the
administration sections, which is the only way 5 and 12 add up.

The planner taught chapter 3 in week 2 and carried its own week 1 and
2 focus lines. Chapters and focus lines now follow lessons.md, and the
spreadsheet is rebuilt. Its README no longer promises two revision
dates for all 41 chapters: 39 get two, the prefaces get none and the
comprehensive reviews get one.
</commit_message>
<xml_diff>
--- a/planner/ict257-study-planner.xlsx
+++ b/planner/ict257-study-planner.xlsx
@@ -1213,7 +1213,7 @@
       </c>
       <c r="E5" s="21" t="inlineStr">
         <is>
-          <t>Getting oriented, the command-line assistant and the shell</t>
+          <t>Getting oriented, system documentation, the command-line assistant and the shell</t>
         </is>
       </c>
       <c r="F5" s="22">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>Getting oriented, the command-line assistant and the shell</t>
+          <t>Getting oriented, system documentation, the command-line assistant and the shell</t>
         </is>
       </c>
       <c r="F6" s="22">
@@ -1305,7 +1305,7 @@
       </c>
       <c r="E7" s="21" t="inlineStr">
         <is>
-          <t>Getting oriented, the command-line assistant and the shell</t>
+          <t>Getting oriented, system documentation, the command-line assistant and the shell</t>
         </is>
       </c>
       <c r="F7" s="22">
@@ -1343,11 +1343,11 @@
         </is>
       </c>
       <c r="D8" s="19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" s="21" t="inlineStr">
         <is>
-          <t>Manual pages, registering systems, the file-system hierarchy and working with files</t>
+          <t>Getting oriented, system documentation, the command-line assistant and the shell</t>
         </is>
       </c>
       <c r="F8" s="22">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E9" s="21" t="inlineStr">
         <is>
-          <t>Manual pages, registering systems, the file-system hierarchy and working with files</t>
+          <t>Registering systems, the file-system hierarchy and working with files</t>
         </is>
       </c>
       <c r="F9" s="22">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="E10" s="21" t="inlineStr">
         <is>
-          <t>Getting oriented, the command-line assistant and the shell</t>
+          <t>Getting oriented, system documentation, the command-line assistant and the shell</t>
         </is>
       </c>
       <c r="F10" s="22">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
-          <t>Manual pages, registering systems, the file-system hierarchy and working with files</t>
+          <t>Registering systems, the file-system hierarchy and working with files</t>
         </is>
       </c>
       <c r="F11" s="22">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="E12" s="21" t="inlineStr">
         <is>
-          <t>Manual pages, registering systems, the file-system hierarchy and working with files</t>
+          <t>Registering systems, the file-system hierarchy and working with files</t>
         </is>
       </c>
       <c r="F12" s="22">

</xml_diff>